<commit_message>
Finalize tested ETL pipeline
</commit_message>
<xml_diff>
--- a/output/Student_Report.xlsx
+++ b/output/Student_Report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1975,16 +1975,44 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>24</v>
+        <v>78</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>C</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Fail</t>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>156</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Mineesh</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>MBA</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>67</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>

</xml_diff>